<commit_message>
Real time notification implemented, roles and privildges code rewritten and the nav bar display changed
</commit_message>
<xml_diff>
--- a/services/drugs.xlsx
+++ b/services/drugs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\Hakeem\e-CLINIC\services\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83296874-3157-46BE-9FD6-67138BC4B532}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A409342-5532-45F3-865A-21BA59914BE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6078,7 +6078,18 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -45808,6 +45819,9 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="B1:B1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>